<commit_message>
Work 21 May 2025
</commit_message>
<xml_diff>
--- a/AtchisonRegime/Outputs/Aust/ASX300/df_regEquityReturns_ASX300.xlsx
+++ b/AtchisonRegime/Outputs/Aust/ASX300/df_regEquityReturns_ASX300.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q544"/>
+  <dimension ref="A1:Q545"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -30853,7 +30853,7 @@
         <v>-0.9726698406613064</v>
       </c>
       <c r="C534" t="n">
-        <v>0.1460332201527155</v>
+        <v>0.1241894196525952</v>
       </c>
       <c r="D534" t="b">
         <v>0</v>
@@ -30910,7 +30910,7 @@
         <v>-0.930850647666511</v>
       </c>
       <c r="C535" t="n">
-        <v>0.2388191536463469</v>
+        <v>0.2339228301603335</v>
       </c>
       <c r="D535" t="b">
         <v>0</v>
@@ -30967,7 +30967,7 @@
         <v>-0.8890737992235942</v>
       </c>
       <c r="C536" t="n">
-        <v>0.2406013064670542</v>
+        <v>0.2370619522653315</v>
       </c>
       <c r="D536" t="b">
         <v>0</v>
@@ -31024,7 +31024,7 @@
         <v>-1.090435517906162</v>
       </c>
       <c r="C537" t="n">
-        <v>0.2007569734303624</v>
+        <v>0.1988546216055985</v>
       </c>
       <c r="D537" t="b">
         <v>0</v>
@@ -31081,7 +31081,7 @@
         <v>-1.28973601261699</v>
       </c>
       <c r="C538" t="n">
-        <v>0.1400914415231331</v>
+        <v>0.1425534339131948</v>
       </c>
       <c r="D538" t="b">
         <v>0</v>
@@ -31138,7 +31138,7 @@
         <v>-1.487030325470401</v>
       </c>
       <c r="C539" t="n">
-        <v>0.08697420027797154</v>
+        <v>0.0881118604449648</v>
       </c>
       <c r="D539" t="b">
         <v>0</v>
@@ -31195,7 +31195,7 @@
         <v>-1.508648286865362</v>
       </c>
       <c r="C540" t="n">
-        <v>0.04458779450515634</v>
+        <v>0.05049734109636209</v>
       </c>
       <c r="D540" t="b">
         <v>0</v>
@@ -31252,7 +31252,7 @@
         <v>-1.530614951002829</v>
       </c>
       <c r="C541" t="n">
-        <v>0.03030594341745388</v>
+        <v>0.05226649969174183</v>
       </c>
       <c r="D541" t="b">
         <v>0</v>
@@ -31309,7 +31309,7 @@
         <v>-1.552867908392353</v>
       </c>
       <c r="C542" t="n">
-        <v>0.04619714416039293</v>
+        <v>0.06685384186450997</v>
       </c>
       <c r="D542" t="b">
         <v>0</v>
@@ -31366,7 +31366,7 @@
         <v>-1.4620752903488</v>
       </c>
       <c r="C543" t="n">
-        <v>0.03127296425735279</v>
+        <v>0.0775006846619135</v>
       </c>
       <c r="D543" t="b">
         <v>0</v>
@@ -31420,10 +31420,10 @@
         <v>45747</v>
       </c>
       <c r="B544" t="n">
-        <v>-1.380584681996217</v>
+        <v>-1.383605099136776</v>
       </c>
       <c r="C544" t="n">
-        <v>0.04765921338260101</v>
+        <v>0.09199325928623918</v>
       </c>
       <c r="D544" t="b">
         <v>0</v>
@@ -31469,6 +31469,63 @@
         <v>144.5879049730617</v>
       </c>
       <c r="Q544" t="n">
+        <v>145.2785989199411</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="2" t="n">
+        <v>45777</v>
+      </c>
+      <c r="B545" t="n">
+        <v>-1.312657793185081</v>
+      </c>
+      <c r="C545" t="n">
+        <v>0.08562355455682437</v>
+      </c>
+      <c r="D545" t="b">
+        <v>0</v>
+      </c>
+      <c r="E545" t="b">
+        <v>1</v>
+      </c>
+      <c r="F545" t="n">
+        <v>-3.3390961965401</v>
+      </c>
+      <c r="G545" t="n">
+        <v>10032235.05484365</v>
+      </c>
+      <c r="H545" t="inlineStr">
+        <is>
+          <t>Type 1: Strengthening CLI &amp; Falling Inflation</t>
+        </is>
+      </c>
+      <c r="I545" t="inlineStr">
+        <is>
+          <t>Type 1</t>
+        </is>
+      </c>
+      <c r="J545" t="n">
+        <v>-3.3390961965401</v>
+      </c>
+      <c r="K545" t="n">
+        <v>0</v>
+      </c>
+      <c r="L545" t="n">
+        <v>0</v>
+      </c>
+      <c r="M545" t="n">
+        <v>0</v>
+      </c>
+      <c r="N545" t="n">
+        <v>1476.400972598866</v>
+      </c>
+      <c r="O545" t="n">
+        <v>275.4740587243287</v>
+      </c>
+      <c r="P545" t="n">
+        <v>144.5879049730617</v>
+      </c>
+      <c r="Q545" t="n">
         <v>145.2785989199411</v>
       </c>
     </row>

</xml_diff>